<commit_message>
docs: user/dev/admin guides, full deploy, promo economics sheet
</commit_message>
<xml_diff>
--- a/docs/biznes/ЭКОНОМИКА.xlsx
+++ b/docs/biznes/ЭКОНОМИКА.xlsx
@@ -11,10 +11,11 @@
     <sheet name="Ввод" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Фикс" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Пакеты" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Калькулятор" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Реклама" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Балансы" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Подписка" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Промо" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Калькулятор" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Реклама" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Балансы" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Подписка" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -568,76 +569,88 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Калькулятор</t>
+          <t>Промо</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Точка безубыточности</t>
+          <t>Скидка % для беты — маржа после GP+НПД</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Реклама</t>
+          <t>Калькулятор</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAC / LTV / пробные</t>
+          <t>Точка безубыточности</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Балансы</t>
+          <t>Реклама</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Журнал пополнений API</t>
+          <t>CAC / LTV / пробные</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Балансы</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Журнал пополнений API</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Подписка</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Черновик планов</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Текст для ассистента:</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>docs/biznes/ЭКОНОМИКА.txt</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Текст для ассистента:</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>docs/biznes/ЭКОНОМИКА.txt §11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Обновлено:</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>10 июля 2026</t>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15 июля 2026</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1057,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Пакеты нот (как на сайте v2.11.9)</t>
+          <t>Пакеты нот (как на сайте v2.11.30)</t>
         </is>
       </c>
     </row>
@@ -1217,6 +1230,274 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Промо для тестеров (GetPlatinum). Жёлтое — меняйте.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Скидка промокода, %</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Перем. себест. 1 ноты ₽ (из Ввод B15)</t>
+        </is>
+      </c>
+      <c r="B4" s="8">
+        <f>Ввод!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GP % + НПД %</t>
+        </is>
+      </c>
+      <c r="B5" s="9">
+        <f>Ввод!B10+Ввод!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Рабочий пол ₽/нота (запас)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Пакет</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Нот</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Цена ₽</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>После скидки ₽</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>₽/нота</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Себест. нот ₽</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Маржа ₽</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>₽/н ≥ пол?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>notes_1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>299</v>
+      </c>
+      <c r="D9" s="8">
+        <f>C9*(1-$B$3)</f>
+        <v/>
+      </c>
+      <c r="E9" s="8">
+        <f>D9/B9</f>
+        <v/>
+      </c>
+      <c r="F9" s="8">
+        <f>B9*$B$4+D9*$B$5</f>
+        <v/>
+      </c>
+      <c r="G9" s="8">
+        <f>D9-F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="10">
+        <f>IF(E9&gt;=$B$6,"ДА","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>notes_3</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>749</v>
+      </c>
+      <c r="D10" s="8">
+        <f>C10*(1-$B$3)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>D10/B10</f>
+        <v/>
+      </c>
+      <c r="F10" s="8">
+        <f>B10*$B$4+D10*$B$5</f>
+        <v/>
+      </c>
+      <c r="G10" s="8">
+        <f>D10-F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="10">
+        <f>IF(E10&gt;=$B$6,"ДА","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>notes_5</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11*(1-$B$3)</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>D11/B11</f>
+        <v/>
+      </c>
+      <c r="F11" s="8">
+        <f>B11*$B$4+D11*$B$5</f>
+        <v/>
+      </c>
+      <c r="G11" s="8">
+        <f>D11-F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="10">
+        <f>IF(E11&gt;=$B$6,"ДА","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>notes_10</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1799</v>
+      </c>
+      <c r="D12" s="8">
+        <f>C12*(1-$B$3)</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>D12/B12</f>
+        <v/>
+      </c>
+      <c r="F12" s="8">
+        <f>B12*$B$4+D12*$B$5</f>
+        <v/>
+      </c>
+      <c r="G12" s="8">
+        <f>D12-F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="10">
+        <f>IF(E12&gt;=$B$6,"ДА","нет")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Рекомендация (текст)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Бета: 30–40% комфортно. 50% ок при малом числе тестеров. &gt;60% на notes_10 — тонкая маржа. 100% только админка ±ноты (маркетинг).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>См. docs/biznes/ЭКОНОМИКА.txt §11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1339,7 +1620,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1448,7 +1729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1609,7 +1890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(econ): real Suno 15cr, GP 3.5%, VPS sizing and promo recalc
</commit_message>
<xml_diff>
--- a/docs/biznes/ЭКОНОМИКА.xlsx
+++ b/docs/biznes/ЭКОНОМИКА.xlsx
@@ -700,7 +700,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Курс USD → RUB</t>
+          <t>Курс USD → RUB (справочно)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -715,11 +715,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Suno + ApiPass, ₽/нота (оценка)</t>
+          <t>Suno, ₽/нота (15 cr, 1000cr=500₽)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.03</v>
+        <v>0.035</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -926,11 +926,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VPS 195.19.20.245</t>
+          <t>VPS (сейчас копейки / заложить рост)</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -941,11 +941,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Домен sozdaipesnu.ru</t>
+          <t>Домен sozdaipesnu.ru (продление/12)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -971,11 +971,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S3 REG.RU</t>
+          <t>S3 REG.RU Object Storage</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -986,11 +986,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Yandex Cloud (мин.)</t>
+          <t>Yandex Cloud (мин./факт)</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1001,11 +1001,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Прочее (мониторинг и т.п.)</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v2.11.42: цены 149 / 375 / 599 / 899
</commit_message>
<xml_diff>
--- a/docs/biznes/ЭКОНОМИКА.xlsx
+++ b/docs/biznes/ЭКОНОМИКА.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ввод" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Фикс" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Пакеты" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Промо" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Калькулятор" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Реклама" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Балансы" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Подписка" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ввод" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Фикс" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пакеты" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Промо" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Калькулятор" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реклама" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Балансы" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Подписка" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1057,7 +1057,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Пакеты нот (как на сайте v2.11.30)</t>
+          <t>Пакеты нот (как на сайте v2.11.42)</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>299</v>
+        <v>149</v>
       </c>
       <c r="D4" s="8">
         <f>C4/B4</f>
@@ -1137,7 +1137,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>749</v>
+        <v>375</v>
       </c>
       <c r="D5" s="8">
         <f>C5/B5</f>
@@ -1166,7 +1166,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1199</v>
+        <v>599</v>
       </c>
       <c r="D6" s="8">
         <f>C6/B6</f>
@@ -1195,7 +1195,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1799</v>
+        <v>899</v>
       </c>
       <c r="D7" s="8">
         <f>C7/B7</f>
@@ -1349,7 +1349,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>299</v>
+        <v>149</v>
       </c>
       <c r="D9" s="8">
         <f>C9*(1-$B$3)</f>
@@ -1382,7 +1382,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>749</v>
+        <v>375</v>
       </c>
       <c r="D10" s="8">
         <f>C10*(1-$B$3)</f>
@@ -1415,7 +1415,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>1199</v>
+        <v>599</v>
       </c>
       <c r="D11" s="8">
         <f>C11*(1-$B$3)</f>
@@ -1448,7 +1448,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>1799</v>
+        <v>899</v>
       </c>
       <c r="D12" s="8">
         <f>C12*(1-$B$3)</f>

</xml_diff>